<commit_message>
data(q3): refresh Origin package and preserve old data
</commit_message>
<xml_diff>
--- a/modules/40_q3/figures/editable/origin_templates/data/20_Si阈值决策阶梯图.xlsx
+++ b/modules/40_q3/figures/editable/origin_templates/data/20_Si阈值决策阶梯图.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据" sheetId="1" r:id="R307a9898de6342c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据" sheetId="1" r:id="Rc488ef6f47264a5c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,32 +13,21 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
-    <x:numFmt numFmtId="200" formatCode="0.00"/>
-    <x:numFmt numFmtId="201" formatCode="0"/>
-    <x:numFmt numFmtId="202" formatCode="0.000000"/>
-    <x:numFmt numFmtId="203" formatCode="@"/>
-  </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF222222"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
-      <x:name val="宋体"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="10"/>
-      <x:color rgb="FFFFFFFF"/>
-      <x:name val="Times New Roman"/>
-    </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:name val="Times New Roman"/>
+      <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
   <x:fills count="3">
@@ -54,181 +43,37 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="10">
+  <x:borders count="2">
     <x:border/>
     <x:border>
-      <x:right style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:right>
-      <x:bottom style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
       <x:left style="thin">
-        <x:color rgb="FFE7EEF5"/>
+        <x:color rgb="FFD9E2F3"/>
       </x:left>
       <x:right style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:right>
-      <x:bottom style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:left>
-      <x:bottom style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
-      <x:right style="thin">
-        <x:color rgb="FFE7EEF5"/>
+        <x:color rgb="FFD9E2F3"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="FFE7EEF5"/>
+        <x:color rgb="FFD9E2F3"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFE7EEF5"/>
+        <x:color rgb="FFD9E2F3"/>
       </x:bottom>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:left>
-      <x:right style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:right>
-      <x:top style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:left>
-      <x:top style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
-      <x:right style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:right>
-      <x:top style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:top>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:left>
-      <x:right style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:right>
-      <x:top style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:top>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:left>
-      <x:top style="thin">
-        <x:color rgb="FFE7EEF5"/>
-      </x:top>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="33">
+  <x:cellXfs count="7">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="203" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="0"/>
-    </x:xf>
-    <x:xf numFmtId="203" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="0"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -432,66 +277,66 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="16" t="str">
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="6" t="str">
         <x:v>判据阈值(%)(X)</x:v>
       </x:c>
-      <x:c r="B1" s="17" t="str">
+      <x:c r="B1" s="6" t="str">
         <x:v>模型选择编码(Y)</x:v>
       </x:c>
-      <x:c r="C1" s="17" t="str">
+      <x:c r="C1" s="6" t="str">
         <x:v>第三束最大比(%)(参考Y)</x:v>
       </x:c>
-      <x:c r="D1" s="18" t="str">
+      <x:c r="D1" s="6" t="str">
         <x:v>编码说明(标签)</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="25" t="n">
+      <x:c r="A2" s="2" t="n">
         <x:v>0.05</x:v>
       </x:c>
-      <x:c r="B2" s="27" t="n">
+      <x:c r="B2" s="2" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C2" s="29" t="n">
-        <x:v>0.0029197278522713195</x:v>
-      </x:c>
-      <x:c r="D2" s="31" t="str">
-        <x:v>0=双光束，1=Airy</x:v>
+      <x:c r="C2" s="2" t="n">
+        <x:v>0.0038824475711443</x:v>
+      </x:c>
+      <x:c r="D2" s="2" t="str">
+        <x:v>0=工程语境记录，不用于Airy/双光束正式选模</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="25" t="n">
+      <x:c r="A3" s="2" t="n">
         <x:v>0.1</x:v>
       </x:c>
-      <x:c r="B3" s="27" t="n">
+      <x:c r="B3" s="2" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C3" s="29" t="n">
-        <x:v>0.0029197278522713195</x:v>
-      </x:c>
-      <x:c r="D3" s="31" t="str">
-        <x:v>0=双光束，1=Airy</x:v>
+      <x:c r="C3" s="2" t="n">
+        <x:v>0.0038824475711443</x:v>
+      </x:c>
+      <x:c r="D3" s="2" t="str">
+        <x:v>0=工程语境记录，不用于Airy/双光束正式选模</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="26" t="n">
+      <x:c r="A4" s="2" t="n">
         <x:v>0.2</x:v>
       </x:c>
-      <x:c r="B4" s="28" t="n">
+      <x:c r="B4" s="2" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C4" s="30" t="n">
-        <x:v>0.0029197278522713195</x:v>
-      </x:c>
-      <x:c r="D4" s="32" t="str">
-        <x:v>0=双光束，1=Airy</x:v>
+      <x:c r="C4" s="2" t="n">
+        <x:v>0.0038824475711443</x:v>
+      </x:c>
+      <x:c r="D4" s="2" t="str">
+        <x:v>0=工程语境记录，不用于Airy/双光束正式选模</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>